<commit_message>
Update Release-Notes.xlsx - Folder inventory updated on Sun Jun 22 00:55:51 UTC 2025
</commit_message>
<xml_diff>
--- a/Release-Notes.xlsx
+++ b/Release-Notes.xlsx
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-06-16 11:43:19 UTC</t>
+          <t>2025-06-22 00:55:50 UTC</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Release-Notes.xlsx - Folder inventory updated on Sun Jun 29 00:57:09 UTC 2025
</commit_message>
<xml_diff>
--- a/Release-Notes.xlsx
+++ b/Release-Notes.xlsx
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-06-22 00:55:50 UTC</t>
+          <t>2025-06-29 00:57:09 UTC</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Release-Notes.xlsx - Folder inventory updated on Sun Jul  6 00:56:23 UTC 2025
</commit_message>
<xml_diff>
--- a/Release-Notes.xlsx
+++ b/Release-Notes.xlsx
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-06-29 00:57:09 UTC</t>
+          <t>2025-07-06 00:56:23 UTC</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Release-Notes.xlsx - Folder inventory updated on Sun Jul 13 00:58:04 UTC 2025
</commit_message>
<xml_diff>
--- a/Release-Notes.xlsx
+++ b/Release-Notes.xlsx
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-07-06 00:56:23 UTC</t>
+          <t>2025-07-13 00:58:03 UTC</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Release-Notes.xlsx - Folder inventory updated on Sun Jul 20 00:59:15 UTC 2025
</commit_message>
<xml_diff>
--- a/Release-Notes.xlsx
+++ b/Release-Notes.xlsx
@@ -2353,7 +2353,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2025-07-13 00:58:03 UTC</t>
+          <t>2025-07-20 00:59:15 UTC</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
     </row>

</xml_diff>